<commit_message>
Restore approved polished My payouts layout and correct handoff r2; preserve shell and stable URLs
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -686,7 +686,44 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="86" customHeight="1">
+      <c r="A18" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="0">
+        <is>
+          <t>Визуальный эталон выплат</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="0">
+        <is>
+          <t>Сравнить с доработанным макетом до передачи</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="0">
+        <is>
+          <t>Карточка баланса/запроса, отдельная история и бейджи из finance-headings-v6. Не подменять их обычной v9-страницей. Общая оболочка прежняя; короткие RU/EN и штатный период сохранены.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G17"/>
+  <autoFilter ref="A1:G18"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Audit all finance mockups, correct handoff instructions and payout navigation, publish byte-matched r3 archives
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -723,7 +723,44 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="86" customHeight="1">
+      <c r="A19" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="0">
+        <is>
+          <t>Комплект и архив</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="0">
+        <is>
+          <t>Сверить опубликованные файлы с ZIP и картой источников</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="0">
+        <is>
+          <t>Все HTML/CSS/JS/ресурсы и документы в архиве совпадают с файлами по ссылкам. Три partial и назначение CSS описаны одинаково во всех инструкциях; активный раздел соответствует экрану.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G18"/>
+  <autoFilter ref="A1:G19"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore original live order, ledger and balance components; retain approved headings and frozen CSS; publish r4
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -760,7 +760,81 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="86" customHeight="1">
+      <c r="A20" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="0">
+        <is>
+          <t>Заказы / Операции / Баланс</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="0">
+        <is>
+          <t>Сравнить вложенные компоненты с текущим сайтом</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr" s="0">
+        <is>
+          <t>Сохранены исходные блоки пользователя, GUID-copy, кредитные/статусные бейджи, логотипы, знаки и цвета сумм, различные иконки и multiple-типы. Не проверять только число столбцов и CSS hashes; нужен прямой просмотр соответствующего сайта и рабочего действия.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="86" customHeight="1">
+      <c r="A21" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="0">
+        <is>
+          <t>Заказы</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="0">
+        <is>
+          <t>Сверить цену и статус заказа</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr" s="0">
+        <is>
+          <t>Цена заказа, число приобретённых кредитов и курс выплаты — независимые данные. Не рассчитывать стоимость заказа через payout-rate. Статусы и значки оплаты берутся из существующей модели/компонента.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G19"/>
+  <autoFilter ref="A1:G21"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align financial range filters with scoped r5 adapter; preserve original customer CSS
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -834,7 +834,44 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="86" customHeight="1">
+      <c r="A22" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="0">
+        <is>
+          <t>Операции / Мой баланс</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr" s="0">
+        <is>
+          <t>Сравнить рамки фильтров суммы, даты и остальных полей</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr" s="0">
+        <is>
+          <t>Внешние рамки и центры на общей оси (локальный допуск0.5CSSpx), без margin15px группы и пустого error-placeholder. Проверить пустое/выбранное состояние, focus и открытый календарь; непустую ошибку не скрывать. Исходные CSS/шрифты и остальная админка сохраняются.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:G22"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Audit remaining balance pages; fix current navigation and preview filters; preserve CSS
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -871,7 +871,81 @@
         </is>
       </c>
     </row>
+    <row r="23" ht="86" customHeight="1">
+      <c r="A23" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="0">
+        <is>
+          <t>Карточка / Реквизиты</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr" s="0">
+        <is>
+          <t>Открыть экран и проверить активное меню</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr" s="0">
+        <is>
+          <t>Единственный aria-current=page и родительский active соответствуют «Мой баланс». Старая метка «Заказы» отсутствует; исходные стили меню не изменены.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="86" customHeight="1">
+      <c r="A24" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="0">
+        <is>
+          <t>Партнёры / автономный preview</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="0">
+        <is>
+          <t>Роль агент; блокировка Нет/Да; сброс</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr" s="0">
+        <is>
+          <t>В демонстрации agent показывает строки1и4, Нет — пять строк, Да — пустую выборку, сброс — пять строк. Фильтрация не меняет геометрию. Этот демо-адаптер на сайт не переносить; там проверить существующий backend-фильтр.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G22"/>
+  <autoFilter ref="A1:G24"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align and compact payout register columns with scoped CSS; preserve financial originals
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -945,7 +945,44 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="86" customHeight="1">
+      <c r="A25" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr" s="0">
+        <is>
+          <t>Реестр выплат</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="0">
+        <is>
+          <t>Сверить ширины и текстовые оси RU/EN; фильтр/сортировка/календарь</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr" s="0">
+        <is>
+          <t>Заголовок и значение числа на одной правой оси; даты по центру, текст слева. Grid≤1060px, локальная прокрутка при рабочей области&lt;1012px. Владелец/статус не растягиваются при фильтре; длинное имя и крупные суммы не скрыты и не перекрывают соседей. Только scoped CSS реестра; остальные CSS/страницы сохранены.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G24"/>
+  <autoFilter ref="A1:G25"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align My payouts history columns with scoped CSS and synchronize Igor package r8
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -982,7 +982,44 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="86" customHeight="1">
+      <c r="A26" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr" s="0">
+        <is>
+          <t>Мои выплаты</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr" s="0">
+        <is>
+          <t>Сверить RU/EN ширины и оси истории, фильтр/сортировку, большой баланс и локальный скролл</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr" s="0">
+        <is>
+          <t>Числа и заголовки справа, даты одинаковой ширины по центру, статус слева. История≤1002px; таблица884px или896px на сенсорной ширине. Без скачков ширин, обрезания сумм/статусов и выхода44px action за ячейку. Все прежние CSS, форма, карточки, реквизиты сохранены.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G26"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix partner narrow date-filter overlap after Astra review; synchronize finance package r9
</commit_message>
<xml_diff>
--- a/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
+++ b/deliveries/balance-ui-20261025-r1/ACCEPTANCE.xlsx
@@ -1019,7 +1019,44 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="86" customHeight="1">
+      <c r="A27" t="inlineStr" s="0">
+        <is>
+          <t>BAL-UI-26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr" s="0">
+        <is>
+          <t>Партнёры: фильтры дат</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr" s="0">
+        <is>
+          <t>360/390/767 CSS px, горизонтальный скролл, дата и сброс</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr" s="0">
+        <is>
+          <t>Три ячейки дат по152px вмещают существующее140px поле и отступы; рамки не перекрывают соседние фильтры. На768px+ исходные120px ячейки. Изменён только отдельный scoped адаптер, исходные CSS и логика сохранены.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr" s="0">
+        <is>
+          <t>НЕ ПРОВЕРЕНО НА САЙТЕ</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr" s="0">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:G27"/>
 </worksheet>
 </file>
</xml_diff>